<commit_message>
added split the template
</commit_message>
<xml_diff>
--- a/source/Transmittal.Reports.OpenXML/Reports/TransmittalSummary.xlsx
+++ b/source/Transmittal.Reports.OpenXML/Reports/TransmittalSummary.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8cb514c15eb25f74/Transmittal Testing/Reports/Style3/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Development\Source\Repos\Transmittal\source\Transmittal.Reports.OpenXML\Reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="47" documentId="8_{9965DD62-E1C7-420B-9F8D-E1A0EC2C1FA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D5F57480-A63E-46C6-9CB9-386B10042344}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{672B0CD7-3443-4A4F-9583-929747B6345A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19260" yWindow="1860" windowWidth="35145" windowHeight="19230" xr2:uid="{606C6374-EA5B-4411-AC94-0D7407AA4B49}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="34185" windowHeight="19650" xr2:uid="{606C6374-EA5B-4411-AC94-0D7407AA4B49}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -184,10 +184,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>